<commit_message>
feat: Complete 2025 Buckman workflow with verification
- Re-run step4 to fix incomplete table generation after reboot
- All depletion tables now fully populated
- Verification: All values within bounds (< 65% YoY change)
  - Total pumping: 1,351.91 AF (-1.5%)
  - Rio Pojoaque: 61.42 AF (+1.0%)
  - Rio Tesuque: 33.65 AF (+0.2%)
  - Otowi: 493.80 AF (+5.1%)
  - La Cienega: 3.92 AF (+4.8%)

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/buckman/output/depletion/TABLE_3_Rio_Pojoaque_Tesuque_2025.xlsx
+++ b/buckman/output/depletion/TABLE_3_Rio_Pojoaque_Tesuque_2025.xlsx
@@ -534,19 +534,19 @@
         <v>40.432</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>0.3041851239669421</v>
+        <v>1.059887603305785</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>40.73618512396695</v>
+        <v>41.49188760330578</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>21.015</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.04165090909090909</v>
+        <v>0.1451900826446281</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>21.05665090909091</v>
+        <v>21.16019008264463</v>
       </c>
     </row>
     <row r="4">
@@ -557,19 +557,19 @@
         <v>39.244</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>2.053114710743802</v>
+        <v>3.286809917355372</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>41.2971147107438</v>
+        <v>42.53080991735537</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>22.333</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.3895953719008264</v>
+        <v>0.6008925619834711</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>22.72259537190082</v>
+        <v>22.93389256198347</v>
       </c>
     </row>
     <row r="5">
@@ -580,19 +580,19 @@
         <v>37.971</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>4.772298842975206</v>
+        <v>5.480429752066116</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>42.7432988429752</v>
+        <v>43.45142975206611</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>23.391</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.9983424793388429</v>
+        <v>1.165586776859504</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>24.38934247933884</v>
+        <v>24.5565867768595</v>
       </c>
     </row>
     <row r="6">
@@ -603,19 +603,19 @@
         <v>36.557</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>6.934258512396694</v>
+        <v>7.319305785123967</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>43.4912585123967</v>
+        <v>43.87630578512397</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>24.227</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>1.58764958677686</v>
+        <v>1.628925619834711</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>25.81464958677686</v>
+        <v>25.85592561983471</v>
       </c>
     </row>
     <row r="7">
@@ -626,19 +626,19 @@
         <v>34.928</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>8.77599867768595</v>
+        <v>9.960039669421487</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>43.70399867768595</v>
+        <v>44.88803966942149</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>24.868</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>2.053894214876033</v>
+        <v>2.163332231404959</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>26.92189421487603</v>
+        <v>27.03133223140496</v>
       </c>
     </row>
     <row r="8">
@@ -649,19 +649,19 @@
         <v>33.112</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>11.59372958677686</v>
+        <v>13.11828099173554</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>44.70572958677686</v>
+        <v>46.23028099173554</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>25.327</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>2.634769586776859</v>
+        <v>2.866909090909091</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>27.96176958677686</v>
+        <v>28.19390909090909</v>
       </c>
     </row>
     <row r="9">
@@ -672,19 +672,19 @@
         <v>31.185</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>14.72497785123967</v>
+        <v>15.9417520661157</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>45.90997785123967</v>
+        <v>47.1267520661157</v>
       </c>
       <c r="E9" s="5" t="n">
         <v>25.615</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>3.336723966942148</v>
+        <v>3.496760330578513</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>28.95172396694215</v>
+        <v>29.11176033057851</v>
       </c>
     </row>
     <row r="10">
@@ -695,19 +695,19 @@
         <v>29.226</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>17.31981619834711</v>
+        <v>18.91001652892562</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>46.54581619834711</v>
+        <v>48.13601652892562</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>25.747</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>3.990345123966942</v>
+        <v>4.278644628099174</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>29.73734512396694</v>
+        <v>30.02564462809917</v>
       </c>
     </row>
     <row r="11">
@@ -718,19 +718,19 @@
         <v>27.296</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>20.29580429752066</v>
+        <v>21.87288595041322</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>47.59180429752066</v>
+        <v>49.16888595041323</v>
       </c>
       <c r="E11" s="5" t="n">
         <v>25.737</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>4.706562644628099</v>
+        <v>4.929203305785124</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>30.4435626446281</v>
+        <v>30.66620330578512</v>
       </c>
     </row>
     <row r="12">
@@ -741,19 +741,19 @@
         <v>25.439</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>23.00992462809917</v>
+        <v>24.14429752066116</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>48.44892462809917</v>
+        <v>49.58329752066116</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>25.608</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>5.438324628099173</v>
+        <v>5.516628099173555</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>31.04632462809917</v>
+        <v>31.12462809917356</v>
       </c>
     </row>
     <row r="13">
@@ -764,19 +764,19 @@
         <v>23.678</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>25.1629547107438</v>
+        <v>26.65646280991736</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>48.8409547107438</v>
+        <v>50.33446280991735</v>
       </c>
       <c r="E13" s="5" t="n">
         <v>25.378</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>6.033042644628099</v>
+        <v>6.153719008264463</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>31.4110426446281</v>
+        <v>31.53171900826446</v>
       </c>
     </row>
     <row r="14">
@@ -787,19 +787,19 @@
         <v>22.028</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>27.82615140495868</v>
+        <v>29.37857851239669</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>49.85415140495868</v>
+        <v>51.40657851239669</v>
       </c>
       <c r="E14" s="5" t="n">
         <v>25.067</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>6.666057520661157</v>
+        <v>6.819768595041323</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>31.73305752066116</v>
+        <v>31.88676859504132</v>
       </c>
     </row>
     <row r="15">
@@ -810,19 +810,19 @@
         <v>20.491</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>30.56001917355372</v>
+        <v>32.25397685950413</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>51.05101917355371</v>
+        <v>52.74497685950413</v>
       </c>
       <c r="E15" s="5" t="n">
         <v>24.691</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>7.301660826446281</v>
+        <v>7.411953719008264</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>31.99266082644628</v>
+        <v>32.10295371900826</v>
       </c>
     </row>
     <row r="16">
@@ -833,19 +833,19 @@
         <v>19.068</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>33.20539636363637</v>
+        <v>34.71421487603306</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>52.27339636363637</v>
+        <v>53.78221487603307</v>
       </c>
       <c r="E16" s="5" t="n">
         <v>24.265</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>7.913803636363637</v>
+        <v>7.956396694214876</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>32.17880363636364</v>
+        <v>32.22139669421487</v>
       </c>
     </row>
     <row r="17">
@@ -856,19 +856,19 @@
         <v>17.753</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>35.86355107438017</v>
+        <v>37.61008264462811</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>53.61655107438017</v>
+        <v>55.36308264462811</v>
       </c>
       <c r="E17" s="5" t="n">
         <v>23.8</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>8.536218842975208</v>
+        <v>8.658644628099175</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>32.33621884297521</v>
+        <v>32.45864462809918</v>
       </c>
     </row>
     <row r="18">
@@ -879,19 +879,19 @@
         <v>16.543</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>39.13994578512397</v>
+        <v>40.57834710743802</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>55.68294578512397</v>
+        <v>57.12134710743802</v>
       </c>
       <c r="E18" s="5" t="n">
         <v>23.308</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>9.302794710743802</v>
+        <v>9.505685950413223</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>32.6107947107438</v>
+        <v>32.81368595041322</v>
       </c>
     </row>
     <row r="19">
@@ -902,10 +902,10 @@
         <v>15.429</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>41.76311801652892</v>
+        <v>41.76311801652893</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>57.19211801652892</v>
+        <v>57.19211801652893</v>
       </c>
       <c r="E19" s="5" t="n">
         <v>22.797</v>
@@ -925,19 +925,19 @@
         <v>14.404</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>42.89697520661157</v>
+        <v>42.778</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>57.30097520661157</v>
+        <v>57.182</v>
       </c>
       <c r="E20" s="5" t="n">
         <v>22.273</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>11.32468561983471</v>
+        <v>11.294</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>33.59768561983471</v>
+        <v>33.567</v>
       </c>
     </row>
     <row r="21">
@@ -948,19 +948,19 @@
         <v>13.462</v>
       </c>
       <c r="C21" s="5" t="n">
-        <v>44.42589818181818</v>
+        <v>44.297</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>57.88789818181819</v>
+        <v>57.759</v>
       </c>
       <c r="E21" s="5" t="n">
         <v>21.743</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>12.00055140495868</v>
+        <v>11.967</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>33.74355140495868</v>
+        <v>33.68</v>
       </c>
     </row>
     <row r="22">
@@ -971,19 +971,19 @@
         <v>12.595</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>46.45149619834711</v>
+        <v>46.32672595041322</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>59.04649619834711</v>
+        <v>58.92172595041322</v>
       </c>
       <c r="E22" s="5" t="n">
         <v>21.212</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>12.74332561983471</v>
+        <v>12.70927338842975</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>33.95532561983471</v>
+        <v>33.92127338842975</v>
       </c>
     </row>
     <row r="23">
@@ -1017,19 +1017,19 @@
         <v>11.061</v>
       </c>
       <c r="C24" s="5" t="n">
-        <v>50.14093685950413</v>
+        <v>50.00541619834711</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>61.20193685950413</v>
+        <v>61.06641619834711</v>
       </c>
       <c r="E24" s="5" t="n">
         <v>20.157</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>13.91288925619835</v>
+        <v>13.87545123966942</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>34.06988925619835</v>
+        <v>34.03245123966942</v>
       </c>
     </row>
     <row r="25">
@@ -1040,19 +1040,19 @@
         <v>10.383</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>51.86255404958678</v>
+        <v>51.72275900826447</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>62.24555404958679</v>
+        <v>62.10575900826447</v>
       </c>
       <c r="E25" s="5" t="n">
         <v>19.639</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>14.56468363636364</v>
+        <v>14.52564099173554</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>34.20368363636364</v>
+        <v>34.16464099173554</v>
       </c>
     </row>
     <row r="26">
@@ -1063,19 +1063,19 @@
         <v>6.151</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>53.22150942148761</v>
+        <v>53.07699173553719</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>59.37250942148761</v>
+        <v>59.22799173553719</v>
       </c>
       <c r="E26" s="5" t="n">
         <v>19.258</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>15.20387504132231</v>
+        <v>15.16288462809917</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>34.46187504132232</v>
+        <v>34.42088462809917</v>
       </c>
     </row>
     <row r="27">
@@ -1109,19 +1109,19 @@
         <v>3.234</v>
       </c>
       <c r="C28" s="5" t="n">
-        <v>54.55799801652893</v>
+        <v>54.40987834710744</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>57.79199801652893</v>
+        <v>57.64387834710745</v>
       </c>
       <c r="E28" s="5" t="n">
         <v>18.276</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>15.98892892561983</v>
+        <v>15.94565157024793</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>34.26492892561983</v>
+        <v>34.22165157024794</v>
       </c>
     </row>
     <row r="29">
@@ -1132,19 +1132,19 @@
         <v>1.775</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>55.87780760330579</v>
+        <v>55.72643504132231</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>57.65280760330579</v>
+        <v>57.50143504132231</v>
       </c>
       <c r="E29" s="5" t="n">
         <v>17.785</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>16.51827768595041</v>
+        <v>16.4737547107438</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>34.30327768595041</v>
+        <v>34.2587547107438</v>
       </c>
     </row>
     <row r="30">
@@ -1155,19 +1155,19 @@
         <v>0.316</v>
       </c>
       <c r="C30" s="5" t="n">
-        <v>56.50542347107438</v>
+        <v>56.35140892561984</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>56.82142347107438</v>
+        <v>56.66740892561985</v>
       </c>
       <c r="E30" s="5" t="n">
         <v>17.295</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>16.9358241322314</v>
+        <v>16.88988495867768</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>34.2308241322314</v>
+        <v>34.18488495867769</v>
       </c>
     </row>
     <row r="31">
@@ -1197,19 +1197,19 @@
       </c>
       <c r="B32" s="5" t="n"/>
       <c r="C32" s="5" t="n">
-        <v>57.67730578512398</v>
+        <v>57.52037950413224</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>57.67730578512398</v>
+        <v>57.52037950413224</v>
       </c>
       <c r="E32" s="5" t="n">
         <v>16.313</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>17.63591008264463</v>
+        <v>17.58813421487603</v>
       </c>
       <c r="G32" s="6" t="n">
-        <v>33.94891008264463</v>
+        <v>33.90113421487603</v>
       </c>
     </row>
     <row r="33">
@@ -1218,19 +1218,19 @@
       </c>
       <c r="B33" s="5" t="n"/>
       <c r="C33" s="5" t="n">
-        <v>58.29216</v>
+        <v>58.13341090909091</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>58.29216</v>
+        <v>58.13341090909091</v>
       </c>
       <c r="E33" s="5" t="n">
         <v>15.822</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>18.02276231404959</v>
+        <v>17.97391140495868</v>
       </c>
       <c r="G33" s="6" t="n">
-        <v>33.84476231404959</v>
+        <v>33.79591140495867</v>
       </c>
     </row>
     <row r="34">
@@ -1239,19 +1239,19 @@
       </c>
       <c r="B34" s="5" t="n"/>
       <c r="C34" s="5" t="n">
-        <v>58.84329520661158</v>
+        <v>58.68303272727272</v>
       </c>
       <c r="D34" s="6" t="n">
-        <v>58.84329520661158</v>
+        <v>58.68303272727272</v>
       </c>
       <c r="E34" s="5" t="n">
         <v>15.331</v>
       </c>
       <c r="F34" s="5" t="n">
-        <v>18.43512</v>
+        <v>18.38521190082645</v>
       </c>
       <c r="G34" s="6" t="n">
-        <v>33.76612</v>
+        <v>33.71621190082645</v>
       </c>
     </row>
     <row r="35">
@@ -1260,10 +1260,10 @@
       </c>
       <c r="B35" s="5" t="n"/>
       <c r="C35" s="5" t="n">
-        <v>59.1537441322314</v>
+        <v>59.15374413223141</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>59.1537441322314</v>
+        <v>59.15374413223141</v>
       </c>
       <c r="E35" s="5" t="n">
         <v>14.841</v>
@@ -1281,19 +1281,19 @@
       </c>
       <c r="B36" s="5" t="n"/>
       <c r="C36" s="5" t="n">
-        <v>59.55741421487603</v>
+        <v>59.39508297520661</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>59.55741421487603</v>
+        <v>59.39508297520661</v>
       </c>
       <c r="E36" s="5" t="n">
         <v>14.35</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>19.23200132231405</v>
+        <v>19.17988363636364</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>33.58200132231405</v>
+        <v>33.52988363636364</v>
       </c>
     </row>
     <row r="37">
@@ -1302,20 +1302,19 @@
       </c>
       <c r="B37" s="5" t="n"/>
       <c r="C37" s="5" t="n">
-        <v>60.0075788429752</v>
+        <v>59.84407338842976</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>60.0075788429752</v>
+        <v>59.84407338842976</v>
       </c>
       <c r="E37" s="5" t="n">
         <v>13.859</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>19.6841494214876</v>
-      </c>
-      <c r="G37" s="6">
-        <f>E37+F37</f>
-        <v/>
+        <v>19.63085355371901</v>
+      </c>
+      <c r="G37" s="6" t="n">
+        <v>33.48985355371901</v>
       </c>
     </row>
     <row r="38">
@@ -1324,20 +1323,19 @@
       </c>
       <c r="B38" s="5" t="n"/>
       <c r="C38" s="5" t="n">
-        <v>60.48815008264463</v>
+        <v>60.32330181818182</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>60.48815008264463</v>
+        <v>60.32330181818182</v>
       </c>
       <c r="E38" s="5" t="n">
         <v>13.368</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>20.17765685950413</v>
-      </c>
-      <c r="G38" s="6">
-        <f>E38+F38</f>
-        <v/>
+        <v>20.12304991735537</v>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v>33.49104991735537</v>
       </c>
     </row>
     <row r="39">
@@ -1357,9 +1355,8 @@
       <c r="F39" s="5" t="n">
         <v>20.70572033057851</v>
       </c>
-      <c r="G39" s="6">
-        <f>E39+F39</f>
-        <v/>
+      <c r="G39" s="6" t="n">
+        <v>33.58272033057851</v>
       </c>
     </row>
     <row r="40">
@@ -1379,9 +1376,8 @@
       <c r="F40" s="5" t="n">
         <v>21.26560462809917</v>
       </c>
-      <c r="G40" s="6">
-        <f>E40+F40</f>
-        <v/>
+      <c r="G40" s="6" t="n">
+        <v>33.65260462809917</v>
       </c>
     </row>
     <row r="41">
@@ -1401,9 +1397,8 @@
       <c r="F41" s="5" t="n">
         <v>21.8391173553719</v>
       </c>
-      <c r="G41" s="6">
-        <f>E41+F41</f>
-        <v/>
+      <c r="G41" s="6" t="n">
+        <v>33.7351173553719</v>
       </c>
     </row>
     <row r="42">
@@ -1423,9 +1418,8 @@
       <c r="F42" s="5" t="n">
         <v>22.23224925619834</v>
       </c>
-      <c r="G42" s="6">
-        <f>E42+F42</f>
-        <v/>
+      <c r="G42" s="6" t="n">
+        <v>33.63724925619834</v>
       </c>
     </row>
     <row r="43">
@@ -1445,9 +1439,8 @@
       <c r="F43" s="5" t="n">
         <v>22.56505190082645</v>
       </c>
-      <c r="G43" s="6">
-        <f>E43+F43</f>
-        <v/>
+      <c r="G43" s="6" t="n">
+        <v>33.47905190082645</v>
       </c>
     </row>
     <row r="44">
@@ -1467,9 +1460,8 @@
       <c r="F44" s="5" t="n">
         <v>22.91594975206612</v>
       </c>
-      <c r="G44" s="6">
-        <f>E44+F44</f>
-        <v/>
+      <c r="G44" s="6" t="n">
+        <v>33.33994975206612</v>
       </c>
     </row>
     <row r="45">
@@ -1489,9 +1481,8 @@
       <c r="F45" s="5" t="n">
         <v>23.27644958677686</v>
       </c>
-      <c r="G45" s="6">
-        <f>E45+F45</f>
-        <v/>
+      <c r="G45" s="6" t="n">
+        <v>33.20944958677686</v>
       </c>
     </row>
   </sheetData>

</xml_diff>